<commit_message>
update files and figures
</commit_message>
<xml_diff>
--- a/results/section_2_2_table_2025.xlsx
+++ b/results/section_2_2_table_2025.xlsx
@@ -32,37 +32,37 @@
     <t xml:space="preserve">2010-2019</t>
   </si>
   <si>
-    <t xml:space="preserve">2013-2022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023 (projection)</t>
+    <t xml:space="preserve">2014-2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024 (projection)</t>
   </si>
   <si>
     <t xml:space="preserve">GHG</t>
   </si>
   <si>
-    <t xml:space="preserve">31±4.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35±4.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">39±5.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45±5.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">53±5.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">53±5.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">55±5.1</t>
+    <t xml:space="preserve">30.9±4.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34.7±4.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39.3±5.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45.1±5.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">52.9±5.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">53.7±5.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">55.3±5.1</t>
   </si>
   <si>
     <t xml:space="preserve">CO2-FFI</t>
@@ -83,13 +83,13 @@
     <t xml:space="preserve">35.5±2.8</t>
   </si>
   <si>
-    <t xml:space="preserve">36.1±2.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">37.3±3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">37±2.9</t>
+    <t xml:space="preserve">36.4±2.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">37.8±3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38.1±3</t>
   </si>
   <si>
     <t xml:space="preserve">CO2-LULUCF</t>
@@ -110,13 +110,13 @@
     <t xml:space="preserve">4.9±3.4</t>
   </si>
   <si>
-    <t xml:space="preserve">4.3±3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.5±2.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4±2.8</t>
+    <t xml:space="preserve">4.1±2.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.6±2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.4±3.1</t>
   </si>
   <si>
     <t xml:space="preserve">CH4</t>
@@ -137,10 +137,10 @@
     <t xml:space="preserve">8.4±2.5</t>
   </si>
   <si>
-    <t xml:space="preserve">8.6±2.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9±2.7</t>
+    <t xml:space="preserve">8.7±2.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.2±2.7</t>
   </si>
   <si>
     <t xml:space="preserve">N2O</t>
@@ -185,10 +185,10 @@
     <t xml:space="preserve">1.4±0.42</t>
   </si>
   <si>
-    <t xml:space="preserve">1.6±0.48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.8±0.54</t>
+    <t xml:space="preserve">1.6±0.49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.8±0.55</t>
   </si>
 </sst>
 </file>

</xml_diff>